<commit_message>
clean up and extra testing with the new data we recieved
some parts are cleaner, others are creating more questions
</commit_message>
<xml_diff>
--- a/mappings/parameter_e_h_g.xlsx
+++ b/mappings/parameter_e_h_g.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,6 +480,11 @@
           <t>hoedanigheid_code</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>eenheid_code</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -530,6 +535,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -580,6 +590,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -630,6 +645,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -680,6 +700,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -730,6 +755,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -777,7 +807,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -827,7 +862,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -877,7 +917,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -930,6 +975,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -980,6 +1030,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1030,6 +1085,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1080,6 +1140,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1130,6 +1195,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1180,6 +1250,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1230,6 +1305,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1280,6 +1360,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1330,6 +1415,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1380,6 +1470,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1419,7 +1514,12 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -1472,6 +1572,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1522,6 +1627,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1572,6 +1682,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1622,6 +1737,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1672,6 +1792,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1719,7 +1844,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1899,12 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1954,12 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -1869,7 +2009,12 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -1922,6 +2067,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1972,6 +2122,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2022,6 +2177,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2072,6 +2232,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2119,7 +2284,12 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -2172,6 +2342,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2222,6 +2397,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2272,6 +2452,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2322,6 +2507,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2372,6 +2562,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2422,6 +2617,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2472,6 +2672,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2522,6 +2727,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2572,6 +2782,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2622,6 +2837,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2672,6 +2892,11 @@
           <t>nf</t>
         </is>
       </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>mg/l</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2722,6 +2947,11 @@
           <t>Nnf</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>mg/l</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2772,6 +3002,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2822,6 +3057,11 @@
           <t>nf</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2872,6 +3112,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2922,6 +3167,11 @@
           <t>nf</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2972,6 +3222,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3022,6 +3277,11 @@
           <t>nf</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3072,6 +3332,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3122,6 +3387,11 @@
           <t>nf</t>
         </is>
       </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3172,6 +3442,11 @@
           <t>nf</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3222,6 +3497,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3272,6 +3552,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3322,6 +3607,11 @@
           <t>nf</t>
         </is>
       </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3372,6 +3662,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3422,6 +3717,11 @@
           <t>nf</t>
         </is>
       </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3472,6 +3772,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3522,6 +3827,11 @@
           <t>nf</t>
         </is>
       </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3572,6 +3882,11 @@
           <t>Pnf</t>
         </is>
       </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>mg/l</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3622,6 +3937,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3669,7 +3989,12 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -3722,6 +4047,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3772,6 +4102,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3822,6 +4157,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3872,6 +4212,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3919,7 +4264,12 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -3972,6 +4322,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -4022,6 +4377,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -4072,6 +4432,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -4122,6 +4487,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -4172,6 +4542,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -4222,6 +4597,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -4272,6 +4652,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ng/l</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -4314,6 +4699,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -4353,7 +4743,12 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4790,12 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4837,12 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4884,12 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4931,12 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4986,12 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -4621,7 +5041,12 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -4671,7 +5096,12 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -4724,6 +5154,11 @@
           <t>NVT</t>
         </is>
       </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ug/l</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4771,7 +5206,12 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>OPGLT</t>
+          <t>NVT</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ug/l</t>
         </is>
       </c>
     </row>
@@ -4822,6 +5262,11 @@
       <c r="J89" t="inlineStr">
         <is>
           <t>NVT</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>mg/l</t>
         </is>
       </c>
     </row>
@@ -4836,7 +5281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4890,6 +5335,11 @@
           <t>hoedanigheid_code</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>eenheid_code</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -4916,6 +5366,7 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -4954,6 +5405,7 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -4992,6 +5444,7 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -5030,6 +5483,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -5060,6 +5514,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -5090,6 +5545,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -5120,6 +5576,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -5150,6 +5607,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -5172,6 +5630,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -5194,6 +5653,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -5224,6 +5684,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -5254,6 +5715,7 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -5284,6 +5746,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -5314,6 +5777,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -5344,6 +5808,7 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -5374,6 +5839,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -5404,6 +5870,7 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -5434,6 +5901,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -5460,6 +5928,7 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -5486,6 +5955,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -5516,6 +5986,7 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -5542,6 +6013,7 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -5580,6 +6052,7 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -5618,6 +6091,7 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -5656,6 +6130,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -5686,6 +6161,7 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -5716,6 +6192,7 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -5746,6 +6223,7 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -5776,6 +6254,7 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -5806,6 +6285,7 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -5844,6 +6324,7 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -5870,6 +6351,7 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -5908,6 +6390,7 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -5930,6 +6413,7 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -5952,6 +6436,7 @@
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -5982,6 +6467,7 @@
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -6008,6 +6494,7 @@
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -6038,6 +6525,7 @@
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6070,6 +6558,7 @@
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -6094,6 +6583,7 @@
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6118,6 +6608,7 @@
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -6142,6 +6633,7 @@
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -6158,6 +6650,7 @@
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -6174,6 +6667,7 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -6198,6 +6692,7 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -6219,6 +6714,7 @@
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
@@ -6239,6 +6735,7 @@
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
@@ -6251,6 +6748,7 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>